<commit_message>
Fix patent table layout, footer 报告信息, team_read=4 integrity
Layout: colgroup label column ~132px, full-width figure rows, nested
event tables auto layout; content before footer; no top count strip; TOC
search + short sidebar header.

Data: EVIDENCE-READ-RULING-COMBINED locks team_read=4; apply_read_ruling +
audit_data_integrity; merge_evidence_r2 counts team_independent_read only.
AUTOMATION.md three honest labels. No mass figure PDF restore (await mapping PR).

Figures policy: reserved aspect-ratio on lazy images to reduce layout jump.

Co-authored-by: Chuqin Z <Chuqonu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ledger/patents.xlsx
+++ b/ledger/patents.xlsx
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -707,7 +707,7 @@
     <col width="48" customWidth="1" min="22" max="22"/>
     <col width="21" customWidth="1" min="23" max="23"/>
     <col width="15" customWidth="1" min="24" max="24"/>
-    <col width="19" customWidth="1" min="25" max="25"/>
+    <col width="28" customWidth="1" min="25" max="25"/>
     <col width="20" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
@@ -3621,11 +3621,7 @@
       </c>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>证据复核 r2：权利要求与摘要</t>
-        </is>
-      </c>
+      <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr">
         <is>
           <t>evidence-review-r2</t>
@@ -4634,11 +4630,7 @@
       </c>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>证据复核 r2：权利要求与摘要</t>
-        </is>
-      </c>
+      <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr">
         <is>
           <t>evidence-review-r2</t>
@@ -4764,11 +4756,7 @@
       </c>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>证据复核 r2：权利要求与摘要</t>
-        </is>
-      </c>
+      <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr">
         <is>
           <t>evidence-review-r2</t>
@@ -5526,11 +5514,7 @@
       </c>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr">
-        <is>
-          <t>证据复核 r2：权利要求与摘要</t>
-        </is>
-      </c>
+      <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr">
         <is>
           <t>evidence-review-r2</t>
@@ -5656,11 +5640,7 @@
       </c>
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>证据复核 r2：权利要求与摘要</t>
-        </is>
-      </c>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr">
         <is>
           <t>evidence-review-r2</t>
@@ -7427,7 +7407,7 @@
       <c r="X53" t="inlineStr"/>
       <c r="Y53" t="inlineStr">
         <is>
-          <t>证据复核 r2：权利要求与摘要</t>
+          <t>Gate③ 证据复核：权利要求级阅读（EPI 四件）</t>
         </is>
       </c>
       <c r="Z53" t="inlineStr">
@@ -7557,7 +7537,7 @@
       <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>证据复核 r2：权利要求与摘要</t>
+          <t>Gate③ 证据复核：权利要求级阅读（EPI 四件）</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr">
@@ -8949,7 +8929,7 @@
       <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr">
         <is>
-          <t>证据复核 r2：权利要求与摘要</t>
+          <t>Gate③ 证据复核：权利要求级阅读（EPI 四件）</t>
         </is>
       </c>
       <c r="Z65" t="inlineStr">
@@ -15923,7 +15903,7 @@
       <c r="X120" t="inlineStr"/>
       <c r="Y120" t="inlineStr">
         <is>
-          <t>证据复核 r2：权利要求与摘要</t>
+          <t>Gate③ 证据复核：权利要求级阅读（EPI 四件）</t>
         </is>
       </c>
       <c r="Z120" t="inlineStr">

</xml_diff>

<commit_message>
Apply figure restore to report.json and stamp asset URLs
- restore_reference_figures.py --apply: 130 refs with assets/figures/recovered paths
- counts.figures_available=130; --check exit 0
- Re-stamp index.html + asset-versions.json for new report.json hash

Co-authored-by: Chuqin Z <Chuqonu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ledger/patents.xlsx
+++ b/ledger/patents.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -670,10 +670,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>counts.figures_available</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>counts.figures_pending</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Empty months ≠ zero hits. 2025-09 paused. No zero-omission claim.</t>
         </is>
@@ -23645,11 +23665,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>publication</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>

</xml_diff>

<commit_message>
Hygiene: prune stale pending_or_related to CN122564748A only
Remove promoted/excluded IDs from live pending queue and align
EVIDENCE-REVIEW r2 + sprint/read ruling mirrors. Add prune script,
rebuild ledger xlsx, and stamp report.json cache version.

Co-authored-by: Chuqin Z <Chuqonu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ledger/patents.xlsx
+++ b/ledger/patents.xlsx
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -23821,7 +23821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL6"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23834,9 +23834,9 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="48" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
@@ -23852,14 +23852,14 @@
     <col width="10" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="19" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
     <col width="20" customWidth="1" min="30" max="30"/>
     <col width="23" customWidth="1" min="31" max="31"/>
     <col width="18" customWidth="1" min="32" max="32"/>
     <col width="13" customWidth="1" min="33" max="33"/>
     <col width="48" customWidth="1" min="34" max="34"/>
     <col width="48" customWidth="1" min="35" max="35"/>
-    <col width="28" customWidth="1" min="36" max="36"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
     <col width="21" customWidth="1" min="38" max="38"/>
   </cols>
@@ -24184,17 +24184,17 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>US20260066234A1</t>
+          <t>CN122564748A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>US20260066234A1</t>
+          <t>CN122564748A</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -24204,7 +24204,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -24213,19 +24213,19 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>等离子体增强外延沉积腔室</t>
+          <t>消除外延腔首片膜厚异常的方法</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Applied Materials, Inc.</t>
+          <t>江苏天芯微半导体设备有限公司</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -24254,283 +24254,21 @@
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>已升格 2026-03 主表 core 并计 team_read（r2）；保留队列记录。</t>
+          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>证据复核 r2：独立检索命中但技术边界（等离子体增强外延 vs 纯 preclean/EPI 主线）与同族引用关系待核；未升格为独立新纳入。基线条目中仅作同族附图引用，不重复升格。</t>
+          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>promoted_core_team_read</t>
+          <t>pending_not_promoted</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>US12757451B2</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>US12757451B2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>（公开文献待核实）US12757451B2</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>independent_search</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>证据复核 r2：独立检索列出，但公开日/全文在复核时未能从官方可访问源稳定取得（Google Patents 404）；保留待核，不入主表。</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>公开号 kind/日期未核实；不得默认 A1 公开。</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>pending_verify_publication</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>WO2026084898A1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>WO2026084898A1</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>publication</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>控制含硅外延材料中的自掺杂</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Applied Materials, Inc.</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>imported baseline</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>reference_report</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>证据复核 r2：已在基线主表（imported baseline）。独立检索侧列为待核项系同族/自掺杂边界复核，不升级为独立新发现。</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>证据复核 r2：已在基线主表（imported baseline）。独立检索侧列为待核项系同族/自掺杂边界复核，不升级为独立新发现。</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>pending_not_promoted</t>
-        </is>
-      </c>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CN122564748A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CN122564748A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>publication</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>消除外延腔首片膜厚异常的方法</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>江苏天芯微半导体设备有限公司</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>independent_search</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>pending_not_promoted</t>
-        </is>
-      </c>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24591,13 +24329,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
@@ -24721,32 +24459,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-US12765027B2</t>
-        </is>
-      </c>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:40:17Z</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>pending-queue-hygiene</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>prune_pending_or_related</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Removed promoted/excluded from queue: US20260066234A1, US12757451B2, WO2026084898A1</t>
         </is>
       </c>
     </row>
@@ -24758,7 +24492,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-US20260313994A1</t>
+          <t>2026-10-US12765027B2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -24790,7 +24524,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-US12757647B2</t>
+          <t>2026-10-US20260313994A1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -24822,27 +24556,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-US12757648B2</t>
+          <t>2026-10-US12757647B2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-20T10:37:42Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>sprint-gap-a</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>content_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -24854,27 +24588,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-US20260304810A1</t>
+          <t>2026-10-US12757648B2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>sprint-gap-a</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>content_add</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>
       </c>
     </row>
@@ -24886,7 +24620,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-US12727402B2</t>
+          <t>2026-10-US20260304810A1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -24918,7 +24652,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-US20260275525A1</t>
+          <t>2026-09-US12727402B2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -24950,7 +24684,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-US20260282506A1</t>
+          <t>2026-09-US20260275525A1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -24982,7 +24716,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-US20260282794A1</t>
+          <t>2026-09-US20260282506A1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -25014,7 +24748,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-US12745604B2</t>
+          <t>2026-09-US20260282794A1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -25046,7 +24780,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-US20260293620A1</t>
+          <t>2026-09-US12745604B2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -25078,7 +24812,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-TWI939895B</t>
+          <t>2026-09-US20260293620A1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -25110,7 +24844,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-US12740346B2</t>
+          <t>2026-09-TWI939895B</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -25142,7 +24876,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-US12698570B2</t>
+          <t>2026-09-US12740346B2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -25174,7 +24908,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-US12701762B2</t>
+          <t>2026-08-US12698570B2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -25206,7 +24940,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-US12707938B2</t>
+          <t>2026-08-US12701762B2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -25238,7 +24972,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-US20260250878A1</t>
+          <t>2026-08-US12707938B2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -25270,7 +25004,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-US12701931B2</t>
+          <t>2026-08-US20260250878A1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -25302,7 +25036,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-US20260206272A1</t>
+          <t>2026-08-US12701931B2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -25334,7 +25068,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-US12692621B2</t>
+          <t>2026-07-US20260206272A1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -25366,7 +25100,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-US12696707B2</t>
+          <t>2026-07-US12692621B2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -25398,7 +25132,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-US12680191B2</t>
+          <t>2026-07-US12696707B2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -25430,27 +25164,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-TW202628839A</t>
+          <t>2026-07-US12680191B2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25462,27 +25196,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-06-US20260152871A1</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25494,7 +25228,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-US12652840B2</t>
+          <t>2026-06-US20260152871A1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -25526,7 +25260,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-06-US12655537B2</t>
+          <t>2026-06-US12652840B2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -25558,7 +25292,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-06-US12660266B2</t>
+          <t>2026-06-US12655537B2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -25590,7 +25324,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-06-JP7882130B2</t>
+          <t>2026-06-US12660266B2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -25622,7 +25356,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-06-US12672330B2</t>
+          <t>2026-06-JP7882130B2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -25654,7 +25388,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-06-US20260164725A1</t>
+          <t>2026-06-US12672330B2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -25686,27 +25420,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-06-CN122294515A</t>
+          <t>2026-06-US20260164725A1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25718,7 +25452,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-06-US12660522B2</t>
+          <t>2026-06-CN122294515A</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -25750,27 +25484,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-05-US12628600B2</t>
+          <t>2026-06-US12660522B2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25782,7 +25516,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-05-US12628600B2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -25819,22 +25553,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25846,27 +25580,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-US20260143977A1</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
         </is>
       </c>
     </row>
@@ -25878,7 +25612,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-WO2026101868A1</t>
+          <t>2026-05-US20260143977A1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -25910,7 +25644,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-05-US20260150594A1</t>
+          <t>2026-05-WO2026101868A1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -25942,27 +25676,27 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-CN122069948A</t>
+          <t>2026-05-US20260150594A1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25974,7 +25708,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-WO2026096517A1</t>
+          <t>2026-05-CN122069948A</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -26006,27 +25740,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-04-US20260092399A1</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26038,7 +25772,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-04-JP2026512448A</t>
+          <t>2026-04-US20260092399A1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -26070,7 +25804,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-04-KR102954223B1</t>
+          <t>2026-04-JP2026512448A</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -26102,7 +25836,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-04-WO2026079031A1</t>
+          <t>2026-04-KR102954223B1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -26134,7 +25868,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-04-WO2026084898A1</t>
+          <t>2026-04-WO2026079031A1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -26166,7 +25900,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-04-US20260123349A1</t>
+          <t>2026-04-WO2026084898A1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -26198,7 +25932,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-04-US12595587B2</t>
+          <t>2026-04-US20260123349A1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -26230,7 +25964,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-03-US20260068564A1</t>
+          <t>2026-04-US12595587B2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -26262,7 +25996,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-03-US20260076125A1</t>
+          <t>2026-03-US20260068564A1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -26294,7 +26028,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-03-WO2026055216A1</t>
+          <t>2026-03-US20260076125A1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -26326,7 +26060,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-03-KR20260039926A</t>
+          <t>2026-03-WO2026055216A1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -26358,7 +26092,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-03-US20260090293A1</t>
+          <t>2026-03-KR20260039926A</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -26390,7 +26124,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-03-JP2026510085A</t>
+          <t>2026-03-US20260090293A1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -26422,27 +26156,27 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-03-US20260071979A1</t>
+          <t>2026-03-JP2026510085A</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26454,7 +26188,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-03-CN121693111A</t>
+          <t>2026-03-US20260071979A1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -26486,27 +26220,27 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-03-US20260066234A1</t>
+          <t>2026-03-CN121693111A</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>read-ruling-r2</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>promote_core_team_read</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26518,27 +26252,27 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-02-US12540400B2</t>
+          <t>2026-03-US20260066234A1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T12:00:00Z</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>read-ruling-r2</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>promote_core_team_read</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
         </is>
       </c>
     </row>
@@ -26550,7 +26284,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-02-US20260043170A1</t>
+          <t>2026-02-US12540400B2</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -26582,7 +26316,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-02-US20260047358A1</t>
+          <t>2026-02-US20260043170A1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -26614,7 +26348,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-02-WO2026035639A1</t>
+          <t>2026-02-US20260047358A1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -26646,7 +26380,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-02-CN121519154A</t>
+          <t>2026-02-WO2026035639A1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -26678,7 +26412,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-02-US12557185B2</t>
+          <t>2026-02-CN121519154A</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -26710,7 +26444,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-02-US20260049767A1</t>
+          <t>2026-02-US12557185B2</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -26742,7 +26476,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-02-US12564001B2</t>
+          <t>2026-02-US20260049767A1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -26774,7 +26508,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-US12564001B2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -26811,22 +26545,22 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26838,27 +26572,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-02-US20260035835A1</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
         </is>
       </c>
     </row>
@@ -26870,27 +26604,27 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-02-US20260055532A1</t>
+          <t>2026-02-US20260035835A1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26902,27 +26636,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-01-WO2026005974A1</t>
+          <t>2026-02-US20260055532A1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26934,7 +26668,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-01-US20260009155A1</t>
+          <t>2026-01-WO2026005974A1</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -26966,7 +26700,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-01-US20260009155A1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -27003,22 +26737,22 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27030,27 +26764,27 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-01-US20260015766A1</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
         </is>
       </c>
     </row>
@@ -27062,7 +26796,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-01-KR102915695B1</t>
+          <t>2026-01-US20260015766A1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -27094,7 +26828,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-01-WO2026016396A1</t>
+          <t>2026-01-KR102915695B1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -27126,7 +26860,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-01-WO2026024419A1</t>
+          <t>2026-01-WO2026016396A1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -27158,7 +26892,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-01-KR102918757B1</t>
+          <t>2026-01-WO2026024419A1</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -27190,7 +26924,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-01-US20260026275A1</t>
+          <t>2026-01-KR102918757B1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -27222,7 +26956,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2025-12-KR20250168533A</t>
+          <t>2026-01-US20260026275A1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -27254,7 +26988,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2025-12-US20250379096A1</t>
+          <t>2025-12-KR20250168533A</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -27286,7 +27020,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2025-12-US20250385089A1</t>
+          <t>2025-12-US20250379096A1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -27318,7 +27052,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2025-12-US20250385122A1</t>
+          <t>2025-12-US20250385089A1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -27350,7 +27084,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2025-12-US12503791B2</t>
+          <t>2025-12-US20250385122A1</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -27382,7 +27116,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2025-12-KR102904356B1</t>
+          <t>2025-12-US12503791B2</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -27414,7 +27148,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2025-12-WO2025260942A1</t>
+          <t>2025-12-KR102904356B1</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -27446,7 +27180,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2025-12-US12512362B2</t>
+          <t>2025-12-WO2025260942A1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -27478,7 +27212,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2025-12-US20250369154A1</t>
+          <t>2025-12-US12512362B2</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -27510,7 +27244,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2025-11-KR102886069B1</t>
+          <t>2025-12-US20250369154A1</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -27542,7 +27276,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2025-11-US20250351329A1</t>
+          <t>2025-11-KR102886069B1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -27574,7 +27308,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2025-11-WO2025232199A1</t>
+          <t>2025-11-US20250351329A1</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -27606,7 +27340,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2025-11-TW202544883A</t>
+          <t>2025-11-WO2025232199A1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -27638,7 +27372,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2025-11-KR102888301B1</t>
+          <t>2025-11-TW202544883A</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -27670,7 +27404,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2025-11-US20250358906A1</t>
+          <t>2025-11-KR102888301B1</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -27702,7 +27436,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2025-11-CN120989593A</t>
+          <t>2025-11-US20250358906A1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -27734,7 +27468,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2025-11-CN121002222A</t>
+          <t>2025-11-CN120989593A</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -27766,7 +27500,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2025-11-CN121002231A</t>
+          <t>2025-11-CN121002222A</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -27798,7 +27532,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2025-11-CN121002616A</t>
+          <t>2025-11-CN121002231A</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -27830,7 +27564,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2025-11-CN121002621A</t>
+          <t>2025-11-CN121002616A</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -27862,7 +27596,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2025-11-KR102889785B1</t>
+          <t>2025-11-CN121002621A</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -27894,7 +27628,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2025-11-TWI905596B</t>
+          <t>2025-11-KR102889785B1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -27926,7 +27660,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2025-11-CN223598701U</t>
+          <t>2025-11-TWI905596B</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -27958,7 +27692,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2025-11-US12480223B2</t>
+          <t>2025-11-CN223598701U</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -27990,7 +27724,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2025-11-US12482662B2</t>
+          <t>2025-11-US12480223B2</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -28022,7 +27756,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2025-11-US12484327B2</t>
+          <t>2025-11-US12482662B2</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -28054,7 +27788,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2025-11-JP7776424B2</t>
+          <t>2025-11-US12484327B2</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -28086,7 +27820,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2025-11-DE112021001213B4</t>
+          <t>2025-11-JP7776424B2</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -28118,7 +27852,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2025-11-WO2025244833A1</t>
+          <t>2025-11-DE112021001213B4</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -28150,7 +27884,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2025-10-WO2025225316A1</t>
+          <t>2025-11-WO2025244833A1</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -28182,7 +27916,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2025-10-WO2025222891A1</t>
+          <t>2025-10-WO2025225316A1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -28214,7 +27948,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2025-10-US12454769B2</t>
+          <t>2025-10-WO2025222891A1</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -28246,7 +27980,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2025-10-US20250327211A1</t>
+          <t>2025-10-US12454769B2</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -28278,7 +28012,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2025-10-WO2025220436A1</t>
+          <t>2025-10-US20250327211A1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -28310,7 +28044,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2025-10-WO2025221932A1</t>
+          <t>2025-10-WO2025220436A1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -28342,7 +28076,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2025-10-US20250331222A1</t>
+          <t>2025-10-WO2025221932A1</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -28374,27 +28108,27 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2025-10-US20250327209A1</t>
+          <t>2025-10-US20250331222A1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28406,27 +28140,27 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2025-10-JP7757917B2</t>
+          <t>2025-10-US20250327209A1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -28438,7 +28172,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2025-10-KR20250150601A</t>
+          <t>2025-10-JP7757917B2</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -28470,7 +28204,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2025-10-CN120797198A</t>
+          <t>2025-10-KR20250150601A</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -28502,7 +28236,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2025-10-US20250324699A1</t>
+          <t>2025-10-CN120797198A</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -28534,7 +28268,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2025-10-US12444605B2</t>
+          <t>2025-10-US20250324699A1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -28566,7 +28300,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2025-10-KR102870814B1</t>
+          <t>2025-10-US12444605B2</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -28598,7 +28332,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2025-10-WO2025211045A1</t>
+          <t>2025-10-KR102870814B1</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -28630,7 +28364,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2025-10-JP2025533523A</t>
+          <t>2025-10-WO2025211045A1</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -28662,7 +28396,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2025-10-WO2025204274A1</t>
+          <t>2025-10-JP2025533523A</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -28694,25 +28428,57 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
+          <t>2025-10-WO2025204274A1</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
           <t>2025-10-US20250311241A1</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr">
+      <c r="D130" t="inlineStr">
         <is>
           <t>sprint-gap-a</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>content_add</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
+      <c r="F130" t="inlineStr">
         <is>
           <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>

</xml_diff>

<commit_message>
Pending-queue hygiene: active 待核 = CN122564748A only
Remove promoted/excluded IDs from live pending queue and align
EVIDENCE-REVIEW r2 + sprint/read ruling mirrors. Add prune script,
rebuild ledger xlsx, and stamp report.json cache version.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Chuqin Z <Chuqonu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ledger/patents.xlsx
+++ b/ledger/patents.xlsx
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -23821,7 +23821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL6"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23834,9 +23834,9 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="48" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
@@ -23852,14 +23852,14 @@
     <col width="10" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="19" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
     <col width="20" customWidth="1" min="30" max="30"/>
     <col width="23" customWidth="1" min="31" max="31"/>
     <col width="18" customWidth="1" min="32" max="32"/>
     <col width="13" customWidth="1" min="33" max="33"/>
     <col width="48" customWidth="1" min="34" max="34"/>
     <col width="48" customWidth="1" min="35" max="35"/>
-    <col width="28" customWidth="1" min="36" max="36"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
     <col width="21" customWidth="1" min="38" max="38"/>
   </cols>
@@ -24184,17 +24184,17 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>US20260066234A1</t>
+          <t>CN122564748A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>US20260066234A1</t>
+          <t>CN122564748A</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -24204,7 +24204,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -24213,19 +24213,19 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>等离子体增强外延沉积腔室</t>
+          <t>消除外延腔首片膜厚异常的方法</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Applied Materials, Inc.</t>
+          <t>江苏天芯微半导体设备有限公司</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -24254,283 +24254,21 @@
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>已升格 2026-03 主表 core 并计 team_read（r2）；保留队列记录。</t>
+          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>证据复核 r2：独立检索命中但技术边界（等离子体增强外延 vs 纯 preclean/EPI 主线）与同族引用关系待核；未升格为独立新纳入。基线条目中仅作同族附图引用，不重复升格。</t>
+          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>promoted_core_team_read</t>
+          <t>pending_not_promoted</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>US12757451B2</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>US12757451B2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>（公开文献待核实）US12757451B2</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>independent_search</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>证据复核 r2：独立检索列出，但公开日/全文在复核时未能从官方可访问源稳定取得（Google Patents 404）；保留待核，不入主表。</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>公开号 kind/日期未核实；不得默认 A1 公开。</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>pending_verify_publication</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>WO2026084898A1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>WO2026084898A1</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>publication</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>控制含硅外延材料中的自掺杂</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Applied Materials, Inc.</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>imported baseline</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>reference_report</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>证据复核 r2：已在基线主表（imported baseline）。独立检索侧列为待核项系同族/自掺杂边界复核，不升级为独立新发现。</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>证据复核 r2：已在基线主表（imported baseline）。独立检索侧列为待核项系同族/自掺杂边界复核，不升级为独立新发现。</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>pending_not_promoted</t>
-        </is>
-      </c>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CN122564748A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CN122564748A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>publication</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>消除外延腔首片膜厚异常的方法</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>江苏天芯微半导体设备有限公司</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>independent_search</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>pending_not_promoted</t>
-        </is>
-      </c>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24591,13 +24329,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
@@ -24721,32 +24459,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-US12765027B2</t>
-        </is>
-      </c>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:40:17Z</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>pending-queue-hygiene</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>prune_pending_or_related</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Removed promoted/excluded from queue: US20260066234A1, US12757451B2, WO2026084898A1</t>
         </is>
       </c>
     </row>
@@ -24758,7 +24492,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-US20260313994A1</t>
+          <t>2026-10-US12765027B2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -24790,7 +24524,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-US12757647B2</t>
+          <t>2026-10-US20260313994A1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -24822,27 +24556,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-US12757648B2</t>
+          <t>2026-10-US12757647B2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-20T10:37:42Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>sprint-gap-a</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>content_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -24854,27 +24588,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-US20260304810A1</t>
+          <t>2026-10-US12757648B2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>sprint-gap-a</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>content_add</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>
       </c>
     </row>
@@ -24886,7 +24620,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-US12727402B2</t>
+          <t>2026-10-US20260304810A1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -24918,7 +24652,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-US20260275525A1</t>
+          <t>2026-09-US12727402B2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -24950,7 +24684,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-US20260282506A1</t>
+          <t>2026-09-US20260275525A1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -24982,7 +24716,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-US20260282794A1</t>
+          <t>2026-09-US20260282506A1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -25014,7 +24748,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-US12745604B2</t>
+          <t>2026-09-US20260282794A1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -25046,7 +24780,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-US20260293620A1</t>
+          <t>2026-09-US12745604B2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -25078,7 +24812,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-TWI939895B</t>
+          <t>2026-09-US20260293620A1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -25110,7 +24844,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-US12740346B2</t>
+          <t>2026-09-TWI939895B</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -25142,7 +24876,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-US12698570B2</t>
+          <t>2026-09-US12740346B2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -25174,7 +24908,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-US12701762B2</t>
+          <t>2026-08-US12698570B2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -25206,7 +24940,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-US12707938B2</t>
+          <t>2026-08-US12701762B2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -25238,7 +24972,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-US20260250878A1</t>
+          <t>2026-08-US12707938B2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -25270,7 +25004,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-US12701931B2</t>
+          <t>2026-08-US20260250878A1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -25302,7 +25036,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-US20260206272A1</t>
+          <t>2026-08-US12701931B2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -25334,7 +25068,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-US12692621B2</t>
+          <t>2026-07-US20260206272A1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -25366,7 +25100,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-US12696707B2</t>
+          <t>2026-07-US12692621B2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -25398,7 +25132,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-US12680191B2</t>
+          <t>2026-07-US12696707B2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -25430,27 +25164,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-TW202628839A</t>
+          <t>2026-07-US12680191B2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25462,27 +25196,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-06-US20260152871A1</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25494,7 +25228,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-US12652840B2</t>
+          <t>2026-06-US20260152871A1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -25526,7 +25260,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-06-US12655537B2</t>
+          <t>2026-06-US12652840B2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -25558,7 +25292,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-06-US12660266B2</t>
+          <t>2026-06-US12655537B2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -25590,7 +25324,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-06-JP7882130B2</t>
+          <t>2026-06-US12660266B2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -25622,7 +25356,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-06-US12672330B2</t>
+          <t>2026-06-JP7882130B2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -25654,7 +25388,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-06-US20260164725A1</t>
+          <t>2026-06-US12672330B2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -25686,27 +25420,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-06-CN122294515A</t>
+          <t>2026-06-US20260164725A1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25718,7 +25452,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-06-US12660522B2</t>
+          <t>2026-06-CN122294515A</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -25750,27 +25484,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-05-US12628600B2</t>
+          <t>2026-06-US12660522B2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25782,7 +25516,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-05-US12628600B2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -25819,22 +25553,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25846,27 +25580,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-US20260143977A1</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
         </is>
       </c>
     </row>
@@ -25878,7 +25612,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-WO2026101868A1</t>
+          <t>2026-05-US20260143977A1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -25910,7 +25644,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-05-US20260150594A1</t>
+          <t>2026-05-WO2026101868A1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -25942,27 +25676,27 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-CN122069948A</t>
+          <t>2026-05-US20260150594A1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25974,7 +25708,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-WO2026096517A1</t>
+          <t>2026-05-CN122069948A</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -26006,27 +25740,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-04-US20260092399A1</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26038,7 +25772,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-04-JP2026512448A</t>
+          <t>2026-04-US20260092399A1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -26070,7 +25804,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-04-KR102954223B1</t>
+          <t>2026-04-JP2026512448A</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -26102,7 +25836,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-04-WO2026079031A1</t>
+          <t>2026-04-KR102954223B1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -26134,7 +25868,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-04-WO2026084898A1</t>
+          <t>2026-04-WO2026079031A1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -26166,7 +25900,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-04-US20260123349A1</t>
+          <t>2026-04-WO2026084898A1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -26198,7 +25932,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-04-US12595587B2</t>
+          <t>2026-04-US20260123349A1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -26230,7 +25964,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-03-US20260068564A1</t>
+          <t>2026-04-US12595587B2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -26262,7 +25996,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-03-US20260076125A1</t>
+          <t>2026-03-US20260068564A1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -26294,7 +26028,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-03-WO2026055216A1</t>
+          <t>2026-03-US20260076125A1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -26326,7 +26060,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-03-KR20260039926A</t>
+          <t>2026-03-WO2026055216A1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -26358,7 +26092,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-03-US20260090293A1</t>
+          <t>2026-03-KR20260039926A</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -26390,7 +26124,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-03-JP2026510085A</t>
+          <t>2026-03-US20260090293A1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -26422,27 +26156,27 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-03-US20260071979A1</t>
+          <t>2026-03-JP2026510085A</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26454,7 +26188,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-03-CN121693111A</t>
+          <t>2026-03-US20260071979A1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -26486,27 +26220,27 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-03-US20260066234A1</t>
+          <t>2026-03-CN121693111A</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>read-ruling-r2</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>promote_core_team_read</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26518,27 +26252,27 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-02-US12540400B2</t>
+          <t>2026-03-US20260066234A1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T12:00:00Z</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>read-ruling-r2</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>promote_core_team_read</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
         </is>
       </c>
     </row>
@@ -26550,7 +26284,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-02-US20260043170A1</t>
+          <t>2026-02-US12540400B2</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -26582,7 +26316,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-02-US20260047358A1</t>
+          <t>2026-02-US20260043170A1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -26614,7 +26348,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-02-WO2026035639A1</t>
+          <t>2026-02-US20260047358A1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -26646,7 +26380,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-02-CN121519154A</t>
+          <t>2026-02-WO2026035639A1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -26678,7 +26412,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-02-US12557185B2</t>
+          <t>2026-02-CN121519154A</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -26710,7 +26444,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-02-US20260049767A1</t>
+          <t>2026-02-US12557185B2</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -26742,7 +26476,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-02-US12564001B2</t>
+          <t>2026-02-US20260049767A1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -26774,7 +26508,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-US12564001B2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -26811,22 +26545,22 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26838,27 +26572,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-02-US20260035835A1</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
         </is>
       </c>
     </row>
@@ -26870,27 +26604,27 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-02-US20260055532A1</t>
+          <t>2026-02-US20260035835A1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26902,27 +26636,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-01-WO2026005974A1</t>
+          <t>2026-02-US20260055532A1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26934,7 +26668,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-01-US20260009155A1</t>
+          <t>2026-01-WO2026005974A1</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -26966,7 +26700,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-01-US20260009155A1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -27003,22 +26737,22 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27030,27 +26764,27 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-01-US20260015766A1</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
         </is>
       </c>
     </row>
@@ -27062,7 +26796,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-01-KR102915695B1</t>
+          <t>2026-01-US20260015766A1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -27094,7 +26828,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-01-WO2026016396A1</t>
+          <t>2026-01-KR102915695B1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -27126,7 +26860,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-01-WO2026024419A1</t>
+          <t>2026-01-WO2026016396A1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -27158,7 +26892,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-01-KR102918757B1</t>
+          <t>2026-01-WO2026024419A1</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -27190,7 +26924,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-01-US20260026275A1</t>
+          <t>2026-01-KR102918757B1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -27222,7 +26956,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2025-12-KR20250168533A</t>
+          <t>2026-01-US20260026275A1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -27254,7 +26988,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2025-12-US20250379096A1</t>
+          <t>2025-12-KR20250168533A</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -27286,7 +27020,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2025-12-US20250385089A1</t>
+          <t>2025-12-US20250379096A1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -27318,7 +27052,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2025-12-US20250385122A1</t>
+          <t>2025-12-US20250385089A1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -27350,7 +27084,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2025-12-US12503791B2</t>
+          <t>2025-12-US20250385122A1</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -27382,7 +27116,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2025-12-KR102904356B1</t>
+          <t>2025-12-US12503791B2</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -27414,7 +27148,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2025-12-WO2025260942A1</t>
+          <t>2025-12-KR102904356B1</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -27446,7 +27180,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2025-12-US12512362B2</t>
+          <t>2025-12-WO2025260942A1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -27478,7 +27212,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2025-12-US20250369154A1</t>
+          <t>2025-12-US12512362B2</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -27510,7 +27244,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2025-11-KR102886069B1</t>
+          <t>2025-12-US20250369154A1</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -27542,7 +27276,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2025-11-US20250351329A1</t>
+          <t>2025-11-KR102886069B1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -27574,7 +27308,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2025-11-WO2025232199A1</t>
+          <t>2025-11-US20250351329A1</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -27606,7 +27340,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2025-11-TW202544883A</t>
+          <t>2025-11-WO2025232199A1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -27638,7 +27372,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2025-11-KR102888301B1</t>
+          <t>2025-11-TW202544883A</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -27670,7 +27404,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2025-11-US20250358906A1</t>
+          <t>2025-11-KR102888301B1</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -27702,7 +27436,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2025-11-CN120989593A</t>
+          <t>2025-11-US20250358906A1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -27734,7 +27468,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2025-11-CN121002222A</t>
+          <t>2025-11-CN120989593A</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -27766,7 +27500,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2025-11-CN121002231A</t>
+          <t>2025-11-CN121002222A</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -27798,7 +27532,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2025-11-CN121002616A</t>
+          <t>2025-11-CN121002231A</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -27830,7 +27564,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2025-11-CN121002621A</t>
+          <t>2025-11-CN121002616A</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -27862,7 +27596,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2025-11-KR102889785B1</t>
+          <t>2025-11-CN121002621A</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -27894,7 +27628,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2025-11-TWI905596B</t>
+          <t>2025-11-KR102889785B1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -27926,7 +27660,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2025-11-CN223598701U</t>
+          <t>2025-11-TWI905596B</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -27958,7 +27692,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2025-11-US12480223B2</t>
+          <t>2025-11-CN223598701U</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -27990,7 +27724,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2025-11-US12482662B2</t>
+          <t>2025-11-US12480223B2</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -28022,7 +27756,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2025-11-US12484327B2</t>
+          <t>2025-11-US12482662B2</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -28054,7 +27788,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2025-11-JP7776424B2</t>
+          <t>2025-11-US12484327B2</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -28086,7 +27820,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2025-11-DE112021001213B4</t>
+          <t>2025-11-JP7776424B2</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -28118,7 +27852,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2025-11-WO2025244833A1</t>
+          <t>2025-11-DE112021001213B4</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -28150,7 +27884,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2025-10-WO2025225316A1</t>
+          <t>2025-11-WO2025244833A1</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -28182,7 +27916,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2025-10-WO2025222891A1</t>
+          <t>2025-10-WO2025225316A1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -28214,7 +27948,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2025-10-US12454769B2</t>
+          <t>2025-10-WO2025222891A1</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -28246,7 +27980,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2025-10-US20250327211A1</t>
+          <t>2025-10-US12454769B2</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -28278,7 +28012,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2025-10-WO2025220436A1</t>
+          <t>2025-10-US20250327211A1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -28310,7 +28044,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2025-10-WO2025221932A1</t>
+          <t>2025-10-WO2025220436A1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -28342,7 +28076,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2025-10-US20250331222A1</t>
+          <t>2025-10-WO2025221932A1</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -28374,27 +28108,27 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2025-10-US20250327209A1</t>
+          <t>2025-10-US20250331222A1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28406,27 +28140,27 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2025-10-JP7757917B2</t>
+          <t>2025-10-US20250327209A1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -28438,7 +28172,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2025-10-KR20250150601A</t>
+          <t>2025-10-JP7757917B2</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -28470,7 +28204,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2025-10-CN120797198A</t>
+          <t>2025-10-KR20250150601A</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -28502,7 +28236,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2025-10-US20250324699A1</t>
+          <t>2025-10-CN120797198A</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -28534,7 +28268,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2025-10-US12444605B2</t>
+          <t>2025-10-US20250324699A1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -28566,7 +28300,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2025-10-KR102870814B1</t>
+          <t>2025-10-US12444605B2</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -28598,7 +28332,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2025-10-WO2025211045A1</t>
+          <t>2025-10-KR102870814B1</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -28630,7 +28364,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2025-10-JP2025533523A</t>
+          <t>2025-10-WO2025211045A1</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -28662,7 +28396,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2025-10-WO2025204274A1</t>
+          <t>2025-10-JP2025533523A</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -28694,25 +28428,57 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
+          <t>2025-10-WO2025204274A1</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
           <t>2025-10-US20250311241A1</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr">
+      <c r="D130" t="inlineStr">
         <is>
           <t>sprint-gap-a</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>content_add</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
+      <c r="F130" t="inlineStr">
         <is>
           <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>

</xml_diff>

<commit_message>
Apply Preclean WO/TW figure backfill; clear CN pending (exclude)
Rebased on epi-4 main (69e6079): attach Gate③ hybrid-preclean figures
from PRECLEAN-REPORT-FIGURES-BACKFILL manifest; pending→0 after
CN122564748A exclude disposition. Preserves research_through=2026-10-20
and actually_read=6. Stamp report.json cache.

Co-authored-by: Chuqin Z <Chuqonu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ledger/patents.xlsx
+++ b/ledger/patents.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18">
@@ -3975,7 +3975,7 @@
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr">
@@ -6142,7 +6142,7 @@
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="inlineStr">
@@ -23821,7 +23821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL3"/>
+  <dimension ref="A1:AL2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23853,13 +23853,13 @@
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
-    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
     <col width="23" customWidth="1" min="31" max="31"/>
     <col width="18" customWidth="1" min="32" max="32"/>
     <col width="13" customWidth="1" min="33" max="33"/>
-    <col width="48" customWidth="1" min="34" max="34"/>
-    <col width="48" customWidth="1" min="35" max="35"/>
-    <col width="22" customWidth="1" min="36" max="36"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="27" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
     <col width="21" customWidth="1" min="38" max="38"/>
   </cols>
@@ -24179,96 +24179,6 @@
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CN122564748A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CN122564748A</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>publication</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>消除外延腔首片膜厚异常的方法</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>江苏天芯微半导体设备有限公司</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>independent_search</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>证据复核 r2：关联外延腔首片工艺，但与核心 EPI/preclean 纳入边界需补读权利要求；暂列待核，不入主表为新发现。</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>pending_not_promoted</t>
-        </is>
-      </c>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24329,14 +24239,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="41" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -24487,96 +24397,84 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-10-US12765027B2</t>
-        </is>
-      </c>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:37:57Z</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>epi-4-maintenance</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>empty_incremental_research_through_bump</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>epi-4 实际定时触发 empty incremental (dual-track 0/0/0); research_through 2026-10-19→2026-10-20; team_read unchanged 6; log docs/runs/2026-10-20-epi-4-full-maintenance.md; evidence docs/EVIDENCE-DIFF-2026-10-20-epi-4.json</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-10-US20260313994A1</t>
-        </is>
-      </c>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>preclean-figure-backfill</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>apply_preclean_report_figures</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>WO/TW hybrid-preclean Gate③ figure paths from Preclean backfill manifest.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-10-US12757647B2</t>
-        </is>
-      </c>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>cn-pending-exclude</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>clear_pending_or_related</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Removed from queue (exclude): CN122564748A</t>
         </is>
       </c>
     </row>
@@ -24588,27 +24486,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-US12757648B2</t>
+          <t>2026-10-US12765027B2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-20T10:37:42Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>sprint-gap-a</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>content_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -24620,7 +24518,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-US20260304810A1</t>
+          <t>2026-10-US20260313994A1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -24652,7 +24550,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-US12727402B2</t>
+          <t>2026-10-US12757647B2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -24684,27 +24582,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-US20260275525A1</t>
+          <t>2026-10-US12757648B2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>sprint-gap-a</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>content_add</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>
       </c>
     </row>
@@ -24716,7 +24614,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-US20260282506A1</t>
+          <t>2026-10-US20260304810A1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -24748,7 +24646,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-US20260282794A1</t>
+          <t>2026-09-US12727402B2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -24780,7 +24678,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-US12745604B2</t>
+          <t>2026-09-US20260275525A1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -24812,7 +24710,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-US20260293620A1</t>
+          <t>2026-09-US20260282506A1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -24844,7 +24742,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-TWI939895B</t>
+          <t>2026-09-US20260282794A1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -24876,7 +24774,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-US12740346B2</t>
+          <t>2026-09-US12745604B2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -24908,7 +24806,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-US12698570B2</t>
+          <t>2026-09-US20260293620A1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -24940,7 +24838,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-US12701762B2</t>
+          <t>2026-09-TWI939895B</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -24972,7 +24870,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-US12707938B2</t>
+          <t>2026-09-US12740346B2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -25004,7 +24902,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-US20260250878A1</t>
+          <t>2026-08-US12698570B2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -25036,7 +24934,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-US12701931B2</t>
+          <t>2026-08-US12701762B2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -25068,7 +24966,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-US20260206272A1</t>
+          <t>2026-08-US12707938B2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -25100,7 +24998,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-US12692621B2</t>
+          <t>2026-08-US20260250878A1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -25132,7 +25030,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-US12696707B2</t>
+          <t>2026-08-US12701931B2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -25164,7 +25062,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-US12680191B2</t>
+          <t>2026-07-US20260206272A1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -25196,27 +25094,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-TW202628839A</t>
+          <t>2026-07-US12692621B2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25228,7 +25126,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-US20260152871A1</t>
+          <t>2026-07-US12696707B2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -25260,7 +25158,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-06-US12652840B2</t>
+          <t>2026-07-US12680191B2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -25292,27 +25190,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-06-US12655537B2</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25324,27 +25222,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-06-US12660266B2</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>preclean-figure-backfill</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
         </is>
       </c>
     </row>
@@ -25356,7 +25254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-06-JP7882130B2</t>
+          <t>2026-06-US20260152871A1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -25388,7 +25286,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-06-US12672330B2</t>
+          <t>2026-06-US12652840B2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -25420,7 +25318,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-06-US20260164725A1</t>
+          <t>2026-06-US12655537B2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -25452,27 +25350,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-06-CN122294515A</t>
+          <t>2026-06-US12660266B2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25484,27 +25382,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-06-US12660522B2</t>
+          <t>2026-06-JP7882130B2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25516,7 +25414,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-US12628600B2</t>
+          <t>2026-06-US12672330B2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -25548,7 +25446,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-06-US20260164725A1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -25580,7 +25478,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-06-CN122294515A</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -25595,12 +25493,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25612,27 +25510,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-US20260143977A1</t>
+          <t>2026-06-US12660522B2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25644,7 +25542,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-05-WO2026101868A1</t>
+          <t>2026-05-US12628600B2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -25676,7 +25574,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-US20260150594A1</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -25708,7 +25606,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-CN122069948A</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -25723,12 +25621,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
         </is>
       </c>
     </row>
@@ -25740,27 +25638,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-05-WO2026096517A1</t>
+          <t>2026-05-US20260143977A1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -25772,7 +25670,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-04-US20260092399A1</t>
+          <t>2026-05-WO2026101868A1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -25804,7 +25702,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-04-JP2026512448A</t>
+          <t>2026-05-US20260150594A1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -25836,27 +25734,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-04-KR102954223B1</t>
+          <t>2026-05-CN122069948A</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25868,27 +25766,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-04-WO2026079031A1</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -25900,27 +25798,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-04-WO2026084898A1</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>preclean-figure-backfill</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
         </is>
       </c>
     </row>
@@ -25932,7 +25830,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-04-US20260123349A1</t>
+          <t>2026-04-US20260092399A1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -25964,7 +25862,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-04-US12595587B2</t>
+          <t>2026-04-JP2026512448A</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -25996,7 +25894,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-03-US20260068564A1</t>
+          <t>2026-04-KR102954223B1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -26028,7 +25926,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-03-US20260076125A1</t>
+          <t>2026-04-WO2026079031A1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -26060,7 +25958,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-03-WO2026055216A1</t>
+          <t>2026-04-WO2026084898A1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -26092,7 +25990,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-03-KR20260039926A</t>
+          <t>2026-04-US20260123349A1</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -26124,7 +26022,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-03-US20260090293A1</t>
+          <t>2026-04-US12595587B2</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -26156,7 +26054,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-03-JP2026510085A</t>
+          <t>2026-03-US20260068564A1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -26188,27 +26086,27 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-03-US20260071979A1</t>
+          <t>2026-03-US20260076125A1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26220,27 +26118,27 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-03-CN121693111A</t>
+          <t>2026-03-WO2026055216A1</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26252,27 +26150,27 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-03-US20260066234A1</t>
+          <t>2026-03-KR20260039926A</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>read-ruling-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>promote_core_team_read</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26284,7 +26182,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-02-US12540400B2</t>
+          <t>2026-03-US20260090293A1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -26316,7 +26214,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-02-US20260043170A1</t>
+          <t>2026-03-JP2026510085A</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -26348,27 +26246,27 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-02-US20260047358A1</t>
+          <t>2026-03-US20260071979A1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26380,27 +26278,27 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-02-WO2026035639A1</t>
+          <t>2026-03-CN121693111A</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26412,27 +26310,27 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-02-CN121519154A</t>
+          <t>2026-03-US20260066234A1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T12:00:00Z</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>read-ruling-r2</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>promote_core_team_read</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
         </is>
       </c>
     </row>
@@ -26444,7 +26342,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-02-US12557185B2</t>
+          <t>2026-02-US12540400B2</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -26476,7 +26374,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-02-US20260049767A1</t>
+          <t>2026-02-US20260043170A1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -26508,7 +26406,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-02-US12564001B2</t>
+          <t>2026-02-US20260047358A1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -26540,7 +26438,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-WO2026035639A1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -26572,27 +26470,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-CN121519154A</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26604,7 +26502,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-02-US20260035835A1</t>
+          <t>2026-02-US12557185B2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -26636,27 +26534,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-02-US20260055532A1</t>
+          <t>2026-02-US20260049767A1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26668,7 +26566,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-01-WO2026005974A1</t>
+          <t>2026-02-US12564001B2</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -26700,7 +26598,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-01-US20260009155A1</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -26732,27 +26630,27 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
         </is>
       </c>
     </row>
@@ -26764,27 +26662,27 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-02-US20260035835A1</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26796,27 +26694,27 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-01-US20260015766A1</t>
+          <t>2026-02-US20260055532A1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -26828,7 +26726,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-01-KR102915695B1</t>
+          <t>2026-01-WO2026005974A1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -26860,7 +26758,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-01-WO2026016396A1</t>
+          <t>2026-01-US20260009155A1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -26892,7 +26790,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-01-WO2026024419A1</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -26924,27 +26822,27 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-01-KR102918757B1</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
         </is>
       </c>
     </row>
@@ -26956,7 +26854,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-01-US20260026275A1</t>
+          <t>2026-01-US20260015766A1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -26988,7 +26886,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2025-12-KR20250168533A</t>
+          <t>2026-01-KR102915695B1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -27020,7 +26918,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2025-12-US20250379096A1</t>
+          <t>2026-01-WO2026016396A1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -27052,7 +26950,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2025-12-US20250385089A1</t>
+          <t>2026-01-WO2026024419A1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -27084,7 +26982,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2025-12-US20250385122A1</t>
+          <t>2026-01-KR102918757B1</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -27116,7 +27014,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2025-12-US12503791B2</t>
+          <t>2026-01-US20260026275A1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -27148,7 +27046,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2025-12-KR102904356B1</t>
+          <t>2025-12-KR20250168533A</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -27180,7 +27078,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2025-12-WO2025260942A1</t>
+          <t>2025-12-US20250379096A1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -27212,7 +27110,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2025-12-US12512362B2</t>
+          <t>2025-12-US20250385089A1</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -27244,7 +27142,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2025-12-US20250369154A1</t>
+          <t>2025-12-US20250385122A1</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -27276,7 +27174,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2025-11-KR102886069B1</t>
+          <t>2025-12-US12503791B2</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -27308,7 +27206,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2025-11-US20250351329A1</t>
+          <t>2025-12-KR102904356B1</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -27340,7 +27238,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2025-11-WO2025232199A1</t>
+          <t>2025-12-WO2025260942A1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -27372,7 +27270,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2025-11-TW202544883A</t>
+          <t>2025-12-US12512362B2</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -27404,7 +27302,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2025-11-KR102888301B1</t>
+          <t>2025-12-US20250369154A1</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -27436,7 +27334,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2025-11-US20250358906A1</t>
+          <t>2025-11-KR102886069B1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -27468,7 +27366,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2025-11-CN120989593A</t>
+          <t>2025-11-US20250351329A1</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -27500,7 +27398,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2025-11-CN121002222A</t>
+          <t>2025-11-WO2025232199A1</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -27532,7 +27430,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2025-11-CN121002231A</t>
+          <t>2025-11-TW202544883A</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -27564,7 +27462,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2025-11-CN121002616A</t>
+          <t>2025-11-KR102888301B1</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -27596,7 +27494,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2025-11-CN121002621A</t>
+          <t>2025-11-US20250358906A1</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -27628,7 +27526,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2025-11-KR102889785B1</t>
+          <t>2025-11-CN120989593A</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -27660,7 +27558,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2025-11-TWI905596B</t>
+          <t>2025-11-CN121002222A</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -27692,7 +27590,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2025-11-CN223598701U</t>
+          <t>2025-11-CN121002231A</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -27724,7 +27622,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2025-11-US12480223B2</t>
+          <t>2025-11-CN121002616A</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -27756,7 +27654,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2025-11-US12482662B2</t>
+          <t>2025-11-CN121002621A</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -27788,7 +27686,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2025-11-US12484327B2</t>
+          <t>2025-11-KR102889785B1</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -27820,7 +27718,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2025-11-JP7776424B2</t>
+          <t>2025-11-TWI905596B</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -27852,7 +27750,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2025-11-DE112021001213B4</t>
+          <t>2025-11-CN223598701U</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -27884,7 +27782,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2025-11-WO2025244833A1</t>
+          <t>2025-11-US12480223B2</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -27916,7 +27814,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2025-10-WO2025225316A1</t>
+          <t>2025-11-US12482662B2</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -27948,7 +27846,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2025-10-WO2025222891A1</t>
+          <t>2025-11-US12484327B2</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -27980,7 +27878,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2025-10-US12454769B2</t>
+          <t>2025-11-JP7776424B2</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -28012,7 +27910,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2025-10-US20250327211A1</t>
+          <t>2025-11-DE112021001213B4</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -28044,7 +27942,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2025-10-WO2025220436A1</t>
+          <t>2025-11-WO2025244833A1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -28076,7 +27974,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2025-10-WO2025221932A1</t>
+          <t>2025-10-WO2025225316A1</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -28108,7 +28006,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2025-10-US20250331222A1</t>
+          <t>2025-10-WO2025222891A1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -28140,27 +28038,27 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2025-10-US20250327209A1</t>
+          <t>2025-10-US12454769B2</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28172,7 +28070,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2025-10-JP7757917B2</t>
+          <t>2025-10-US20250327211A1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -28204,7 +28102,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2025-10-KR20250150601A</t>
+          <t>2025-10-WO2025220436A1</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -28236,7 +28134,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2025-10-CN120797198A</t>
+          <t>2025-10-WO2025221932A1</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -28268,7 +28166,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2025-10-US20250324699A1</t>
+          <t>2025-10-US20250331222A1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -28300,27 +28198,27 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2025-10-US12444605B2</t>
+          <t>2025-10-US20250327209A1</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -28332,7 +28230,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2025-10-KR102870814B1</t>
+          <t>2025-10-JP7757917B2</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -28364,7 +28262,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2025-10-WO2025211045A1</t>
+          <t>2025-10-KR20250150601A</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -28396,7 +28294,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2025-10-JP2025533523A</t>
+          <t>2025-10-CN120797198A</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -28428,7 +28326,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2025-10-WO2025204274A1</t>
+          <t>2025-10-US20250324699A1</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -28460,25 +28358,185 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
+          <t>2025-10-US12444605B2</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2025-10-KR102870814B1</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2025-10-WO2025211045A1</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2025-10-JP2025533523A</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2025-10-WO2025204274A1</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
           <t>2025-10-US20250311241A1</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr">
+      <c r="D135" t="inlineStr">
         <is>
           <t>sprint-gap-a</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>content_add</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
+      <c r="F135" t="inlineStr">
         <is>
           <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>

</xml_diff>

<commit_message>
Track A evening R4: USPTO drawing sheets for US12770834B2 + US12768074B2
Add 21 recovered PNGs from image-ppubs PDFs; figures 170→191.
Locks: actually_read=6, research_through=2026-10-20; OG evidence fields unchanged.

Co-authored-by: Chuqin Z <Chuqonu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ledger/patents.xlsx
+++ b/ledger/patents.xlsx
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>170</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18">
@@ -1054,7 +1054,7 @@
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr">
@@ -1206,7 +1206,7 @@
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr">
@@ -25651,7 +25651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -26201,32 +26201,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-10-US12770834B2</t>
-        </is>
-      </c>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-22T01:54:01Z</t>
+          <t>2026-10-22T12:51:05Z</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>morning-epi-overlap-backfill</t>
+          <t>evening-r4-figure-extract</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>include_core_overlap_backfill</t>
+          <t>apply_evening_r4e_uspto_figures</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>EPI-INCREMENTAL-SPRINT-morning-2026-10-22-frozen.json; EVIDENCE-MORNING-DIFF-2026-10-22 PASS_INCREMENTAL</t>
+          <t>US12770834B2+US12768074B2 drawing sheets; pubs=2; actually_read/research_through/team_read untouched by design</t>
         </is>
       </c>
     </row>
@@ -26238,7 +26234,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-US12768074B2</t>
+          <t>2026-10-US12770834B2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -26270,27 +26266,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-US12765027B2</t>
+          <t>2026-10-US12770834B2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-22T12:51:05Z</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-r4-figure-extract</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_uspto_drawing_sheet_figures</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Track A evening R4: 8 real USPTO drawing-sheet PNGs; team_read lock unchanged</t>
         </is>
       </c>
     </row>
@@ -26302,27 +26298,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-US20260313994A1</t>
+          <t>2026-10-US12768074B2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-22T01:54:01Z</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-epi-overlap-backfill</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_overlap_backfill</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>EPI-INCREMENTAL-SPRINT-morning-2026-10-22-frozen.json; EVIDENCE-MORNING-DIFF-2026-10-22 PASS_INCREMENTAL</t>
         </is>
       </c>
     </row>
@@ -26334,27 +26330,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-US12757647B2</t>
+          <t>2026-10-US12768074B2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-22T12:51:05Z</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-r4-figure-extract</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_uspto_drawing_sheet_figures</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Track A evening R4: 13 real USPTO drawing-sheet PNGs; team_read lock unchanged</t>
         </is>
       </c>
     </row>
@@ -26366,27 +26362,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-US12757648B2</t>
+          <t>2026-10-US12765027B2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-20T10:37:42Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>sprint-gap-a</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>content_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26398,27 +26394,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-US12757648B2</t>
+          <t>2026-10-US20260313994A1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26430,27 +26426,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-US12757665B2</t>
+          <t>2026-10-US12757647B2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>include_core_preclean_family</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26462,27 +26458,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-US12757665B2</t>
+          <t>2026-10-US12757648B2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>sprint-gap-a</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>content_add</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Gate③ backfill 6 figures</t>
+          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>
       </c>
     </row>
@@ -26494,27 +26490,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-US20260304810A1</t>
+          <t>2026-10-US12757648B2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -26526,27 +26522,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-US12727402B2</t>
+          <t>2026-10-US12757665B2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_preclean_family</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -26558,27 +26554,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-US20260275525A1</t>
+          <t>2026-10-US12757665B2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 6 figures</t>
         </is>
       </c>
     </row>
@@ -26590,7 +26586,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-US20260282506A1</t>
+          <t>2026-10-US20260304810A1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -26622,7 +26618,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-US20260282794A1</t>
+          <t>2026-09-US12727402B2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -26654,7 +26650,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-US12745604B2</t>
+          <t>2026-09-US20260275525A1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -26686,7 +26682,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-US20260293620A1</t>
+          <t>2026-09-US20260282506A1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -26718,7 +26714,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-TWI939895B</t>
+          <t>2026-09-US20260282794A1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -26750,7 +26746,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-US12740346B2</t>
+          <t>2026-09-US12745604B2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -26782,7 +26778,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-US12698570B2</t>
+          <t>2026-09-US20260293620A1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -26814,7 +26810,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-US12701762B2</t>
+          <t>2026-09-TWI939895B</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -26846,7 +26842,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-US12707938B2</t>
+          <t>2026-09-US12740346B2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -26878,7 +26874,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-US20260250878A1</t>
+          <t>2026-08-US12698570B2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -26910,7 +26906,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-US12701931B2</t>
+          <t>2026-08-US12701762B2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -26942,7 +26938,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-US20260206272A1</t>
+          <t>2026-08-US12707938B2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -26974,7 +26970,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-US12692621B2</t>
+          <t>2026-08-US20260250878A1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -27006,7 +27002,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-US12696707B2</t>
+          <t>2026-08-US12701931B2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -27038,7 +27034,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-US12680191B2</t>
+          <t>2026-07-US20260206272A1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -27070,27 +27066,27 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-TW202628839A</t>
+          <t>2026-07-US12692621B2</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27102,27 +27098,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-TW202628839A</t>
+          <t>2026-07-US12696707B2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-20T10:50:56Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>preclean-figure-backfill</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27134,7 +27130,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-06-JP7882130B2</t>
+          <t>2026-07-US12680191B2</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -27166,27 +27162,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-06-US12672330B2</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27198,27 +27194,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-06-CN122294515A</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>preclean-figure-backfill</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
         </is>
       </c>
     </row>
@@ -27230,27 +27226,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-06-CN122294515A</t>
+          <t>2026-06-JP7882130B2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-20T13:05:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>preclean-cn-figure-stamp</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>attach_depats_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27262,7 +27258,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-06-US12655537B2</t>
+          <t>2026-06-US12672330B2</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -27294,27 +27290,27 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-06-US12660266B2</t>
+          <t>2026-06-CN122294515A</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27326,27 +27322,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-06-US12660522B2</t>
+          <t>2026-06-CN122294515A</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T13:05:00Z</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>preclean-cn-figure-stamp</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>attach_depats_figures</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
         </is>
       </c>
     </row>
@@ -27358,27 +27354,27 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-06-US12660522B2</t>
+          <t>2026-06-US12655537B2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27390,27 +27386,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-06-US12660544B2</t>
+          <t>2026-06-US12660266B2</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>include_core_preclean_family</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27422,27 +27418,27 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-06-US12660544B2</t>
+          <t>2026-06-US12660522B2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Gate③ backfill 6 figures</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27454,27 +27450,27 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-06-US20260164725A1</t>
+          <t>2026-06-US12660522B2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -27486,27 +27482,27 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-06-US12652840B2</t>
+          <t>2026-06-US12660544B2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_preclean_family</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -27518,27 +27514,27 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-06-US20260152871A1</t>
+          <t>2026-06-US12660544B2</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 6 figures</t>
         </is>
       </c>
     </row>
@@ -27550,7 +27546,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-05-US12628600B2</t>
+          <t>2026-06-US20260164725A1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -27582,7 +27578,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-06-US12652840B2</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -27614,27 +27610,27 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-06-US20260152871A1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27646,7 +27642,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-05-US20260143977A1</t>
+          <t>2026-05-US12628600B2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -27678,7 +27674,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-05-WO2026101868A1</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -27710,27 +27706,27 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-05-US20260150594A1</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
         </is>
       </c>
     </row>
@@ -27742,27 +27738,27 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-05-CN122069948A</t>
+          <t>2026-05-US20260143977A1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27774,27 +27770,27 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-05-CN122069948A</t>
+          <t>2026-05-WO2026101868A1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-20T13:05:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>preclean-cn-figure-stamp</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>attach_depats_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27806,27 +27802,27 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-05-WO2026096517A1</t>
+          <t>2026-05-US20260150594A1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27838,27 +27834,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-05-WO2026096517A1</t>
+          <t>2026-05-CN122069948A</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-20T10:50:56Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>preclean-figure-backfill</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27870,27 +27866,27 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-04-US20260092399A1</t>
+          <t>2026-05-CN122069948A</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:05:00Z</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>preclean-cn-figure-stamp</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_depats_figures</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
         </is>
       </c>
     </row>
@@ -27902,27 +27898,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-04-JP2026512448A</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27934,27 +27930,27 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-04-KR102954223B1</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>preclean-figure-backfill</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
         </is>
       </c>
     </row>
@@ -27966,7 +27962,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-04-WO2026079031A1</t>
+          <t>2026-04-US20260092399A1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -27998,7 +27994,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-04-WO2026084898A1</t>
+          <t>2026-04-JP2026512448A</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -28030,7 +28026,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-04-US20260123349A1</t>
+          <t>2026-04-KR102954223B1</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -28062,7 +28058,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-04-US12595587B2</t>
+          <t>2026-04-WO2026079031A1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -28094,7 +28090,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-03-JP2026510085A</t>
+          <t>2026-04-WO2026084898A1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -28126,7 +28122,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-03-US20260090293A1</t>
+          <t>2026-04-US20260123349A1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -28158,27 +28154,27 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-03-US20260090293A1</t>
+          <t>2026-04-US12595587B2</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>label_baseline_preclean_tag</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>US20260090293A1 已 live baseline；补 Preclean 技术标签（claim12），不计晚间新发现。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28190,7 +28186,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-03-KR20260039926A</t>
+          <t>2026-03-JP2026510085A</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -28222,27 +28218,27 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-03-CN121693111A</t>
+          <t>2026-03-US20260090293A1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28254,27 +28250,27 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-03-CN121693111A</t>
+          <t>2026-03-US20260090293A1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-20T12:50:00Z</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>epi-gate3-cn-figure-backfill</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>attach_fig1_depats</t>
+          <t>label_baseline_preclean_tag</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Official drawing page 1/3 → assets/figures/CN121693111A_fig1.png (08612a81…).</t>
+          <t>US20260090293A1 已 live baseline；补 Preclean 技术标签（claim12），不计晚间新发现。</t>
         </is>
       </c>
     </row>
@@ -28286,7 +28282,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-03-US20260076125A1</t>
+          <t>2026-03-KR20260039926A</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -28318,27 +28314,27 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-03-WO2026055216A1</t>
+          <t>2026-03-CN121693111A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -28350,27 +28346,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-03-US20260071979A1</t>
+          <t>2026-03-CN121693111A</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T12:50:00Z</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>epi-gate3-cn-figure-backfill</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>attach_fig1_depats</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Official drawing page 1/3 → assets/figures/CN121693111A_fig1.png (08612a81…).</t>
         </is>
       </c>
     </row>
@@ -28382,27 +28378,27 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-03-US20260071979A1</t>
+          <t>2026-03-US20260076125A1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28414,7 +28410,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-03-US20260068564A1</t>
+          <t>2026-03-WO2026055216A1</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -28446,27 +28442,27 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-03-US20260066234A1</t>
+          <t>2026-03-US20260071979A1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>read-ruling-r2</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>promote_core_team_read</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -28478,7 +28474,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-03-US20260066234A1</t>
+          <t>2026-03-US20260071979A1</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -28510,27 +28506,27 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-03-US20260062803A1</t>
+          <t>2026-03-US20260068564A1</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>include_core_epi</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>EPI-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28542,27 +28538,27 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-03-US20260062803A1</t>
+          <t>2026-03-US20260066234A1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T12:00:00Z</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>read-ruling-r2</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>promote_core_team_read</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Gate③ backfill 2 figures</t>
+          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
         </is>
       </c>
     </row>
@@ -28574,27 +28570,27 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-02-US12540400B2</t>
+          <t>2026-03-US20260066234A1</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -28606,27 +28602,27 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-02-US20260043170A1</t>
+          <t>2026-03-US20260062803A1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_epi</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>EPI-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -28638,27 +28634,27 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-02-US20260047358A1</t>
+          <t>2026-03-US20260062803A1</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 2 figures</t>
         </is>
       </c>
     </row>
@@ -28670,7 +28666,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-02-WO2026035639A1</t>
+          <t>2026-02-US12540400B2</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -28702,7 +28698,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-02-CN121519154A</t>
+          <t>2026-02-US20260043170A1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -28734,7 +28730,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-02-US12557185B2</t>
+          <t>2026-02-US20260047358A1</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -28766,7 +28762,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-02-US20260049767A1</t>
+          <t>2026-02-WO2026035639A1</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -28798,7 +28794,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-02-US12564001B2</t>
+          <t>2026-02-CN121519154A</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -28830,7 +28826,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-US12557185B2</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -28862,27 +28858,27 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-US20260049767A1</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28894,7 +28890,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-02-US20260035835A1</t>
+          <t>2026-02-US12564001B2</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -28926,27 +28922,27 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-02-US20260055532A1</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28958,27 +28954,27 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-02-US20260055532A1</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
         </is>
       </c>
     </row>
@@ -28990,7 +28986,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-01-WO2026024419A1</t>
+          <t>2026-02-US20260035835A1</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -29022,27 +29018,27 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-01-KR102918757B1</t>
+          <t>2026-02-US20260055532A1</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -29054,27 +29050,27 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-01-WO2026016396A1</t>
+          <t>2026-02-US20260055532A1</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -29086,7 +29082,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-01-US20260026275A1</t>
+          <t>2026-01-WO2026024419A1</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -29118,7 +29114,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-01-KR102915695B1</t>
+          <t>2026-01-KR102918757B1</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -29150,27 +29146,27 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-01-KR102916044B1</t>
+          <t>2026-01-WO2026016396A1</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>include_core_preclean_family</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -29182,27 +29178,27 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-01-KR102916044B1</t>
+          <t>2026-01-US20260026275A1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Gate③ backfill 6 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -29214,7 +29210,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-01-US20260015766A1</t>
+          <t>2026-01-KR102915695B1</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -29246,27 +29242,27 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-01-KR102916044B1</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_preclean_family</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -29278,27 +29274,27 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-01-KR102916044B1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
+          <t>Gate③ backfill 6 figures</t>
         </is>
       </c>
     </row>
@@ -29310,7 +29306,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-01-US20260009155A1</t>
+          <t>2026-01-US20260015766A1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -29342,7 +29338,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-01-WO2026005974A1</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -29374,27 +29370,27 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2025-12-KR20250168533A</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
         </is>
       </c>
     </row>
@@ -29406,7 +29402,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2025-12-US20250379096A1</t>
+          <t>2026-01-US20260009155A1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -29438,7 +29434,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2025-12-US20250385089A1</t>
+          <t>2026-01-WO2026005974A1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -29470,7 +29466,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2025-12-US20250385122A1</t>
+          <t>2025-12-KR20250168533A</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -29502,7 +29498,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2025-12-US12503791B2</t>
+          <t>2025-12-US20250379096A1</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -29534,7 +29530,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2025-12-KR102904356B1</t>
+          <t>2025-12-US20250385089A1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -29566,7 +29562,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2025-12-WO2025260942A1</t>
+          <t>2025-12-US20250385122A1</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -29598,7 +29594,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2025-12-US12512362B2</t>
+          <t>2025-12-US12503791B2</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -29630,7 +29626,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2025-12-US20250369154A1</t>
+          <t>2025-12-KR102904356B1</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -29662,7 +29658,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2025-11-KR102886069B1</t>
+          <t>2025-12-WO2025260942A1</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -29694,7 +29690,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2025-11-US20250351329A1</t>
+          <t>2025-12-US12512362B2</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -29726,7 +29722,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2025-11-WO2025232199A1</t>
+          <t>2025-12-US20250369154A1</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -29758,7 +29754,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2025-11-TW202544883A</t>
+          <t>2025-11-KR102886069B1</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -29790,7 +29786,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2025-11-KR102888301B1</t>
+          <t>2025-11-US20250351329A1</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -29822,7 +29818,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2025-11-US20250358906A1</t>
+          <t>2025-11-WO2025232199A1</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -29854,7 +29850,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2025-11-CN120989593A</t>
+          <t>2025-11-TW202544883A</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -29886,7 +29882,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2025-11-CN121002222A</t>
+          <t>2025-11-KR102888301B1</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -29918,7 +29914,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2025-11-CN121002231A</t>
+          <t>2025-11-US20250358906A1</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -29950,7 +29946,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2025-11-CN121002616A</t>
+          <t>2025-11-CN120989593A</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -29982,7 +29978,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2025-11-CN121002621A</t>
+          <t>2025-11-CN121002222A</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -30014,7 +30010,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2025-11-KR102889785B1</t>
+          <t>2025-11-CN121002231A</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -30046,7 +30042,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2025-11-TWI905596B</t>
+          <t>2025-11-CN121002616A</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -30078,7 +30074,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2025-11-CN223598701U</t>
+          <t>2025-11-CN121002621A</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -30110,7 +30106,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2025-11-US12480223B2</t>
+          <t>2025-11-KR102889785B1</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -30142,7 +30138,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2025-11-US12482662B2</t>
+          <t>2025-11-TWI905596B</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -30174,7 +30170,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2025-11-US12484327B2</t>
+          <t>2025-11-CN223598701U</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -30206,7 +30202,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2025-11-JP7776424B2</t>
+          <t>2025-11-US12480223B2</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -30238,7 +30234,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2025-11-DE112021001213B4</t>
+          <t>2025-11-US12482662B2</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -30270,7 +30266,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2025-11-WO2025244833A1</t>
+          <t>2025-11-US12484327B2</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -30302,7 +30298,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2025-10-WO2025225316A1</t>
+          <t>2025-11-JP7776424B2</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -30334,7 +30330,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2025-10-WO2025222891A1</t>
+          <t>2025-11-DE112021001213B4</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -30366,7 +30362,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2025-10-US12454769B2</t>
+          <t>2025-11-WO2025244833A1</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -30398,7 +30394,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2025-10-US20250327211A1</t>
+          <t>2025-10-WO2025225316A1</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -30430,7 +30426,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2025-10-WO2025220436A1</t>
+          <t>2025-10-WO2025222891A1</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -30462,7 +30458,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2025-10-WO2025221932A1</t>
+          <t>2025-10-US12454769B2</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -30494,7 +30490,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2025-10-US20250331222A1</t>
+          <t>2025-10-US20250327211A1</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -30526,27 +30522,27 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2025-10-US20250327209A1</t>
+          <t>2025-10-WO2025220436A1</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -30558,27 +30554,27 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2025-10-US20250327209A1</t>
+          <t>2025-10-WO2025221932A1</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -30590,7 +30586,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2025-10-JP7757917B2</t>
+          <t>2025-10-US20250331222A1</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -30622,27 +30618,27 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2025-10-KR20250150601A</t>
+          <t>2025-10-US20250327209A1</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -30654,27 +30650,27 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2025-10-CN120797198A</t>
+          <t>2025-10-US20250327209A1</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -30686,7 +30682,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2025-10-US20250324699A1</t>
+          <t>2025-10-JP7757917B2</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -30718,7 +30714,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2025-10-US12444605B2</t>
+          <t>2025-10-KR20250150601A</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -30750,7 +30746,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2025-10-KR102870814B1</t>
+          <t>2025-10-CN120797198A</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -30782,7 +30778,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2025-10-WO2025211045A1</t>
+          <t>2025-10-US20250324699A1</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -30814,7 +30810,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2025-10-JP2025533523A</t>
+          <t>2025-10-US12444605B2</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -30846,7 +30842,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2025-10-WO2025204274A1</t>
+          <t>2025-10-KR102870814B1</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -30878,27 +30874,27 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2025-10-US20250311241A1</t>
+          <t>2025-10-WO2025211045A1</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-20T10:37:42Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>sprint-gap-a</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>content_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -30910,25 +30906,121 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
+          <t>2025-10-JP2025533523A</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2025-10-WO2025204274A1</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
           <t>2025-10-US20250311241A1</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>2026-10-20T10:37:42Z</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>sprint-gap-a</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>content_add</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2025-10-US20250311241A1</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
         <is>
           <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr">
+      <c r="D170" t="inlineStr">
         <is>
           <t>morning-gate3-figures</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr">
+      <c r="E170" t="inlineStr">
         <is>
           <t>attach_gate3_family_figures</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
+      <c r="F170" t="inlineStr">
         <is>
           <t>Gate③ backfill 1 figures</t>
         </is>

</xml_diff>

<commit_message>
Track A: figures for US12770834B2 + US12768074B2 (#35)
Evening R4e: 21 USPTO drawing sheets; figures 170→191; Fig.1 display_rotation=0; stamp 61d861b8698e; actually_read=6; research_through=2026-10-20.
</commit_message>
<xml_diff>
--- a/ledger/patents.xlsx
+++ b/ledger/patents.xlsx
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>170</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18">
@@ -1054,7 +1054,7 @@
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr">
@@ -1206,7 +1206,7 @@
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr">
@@ -25651,7 +25651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -26201,32 +26201,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-10-US12770834B2</t>
-        </is>
-      </c>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-22T01:54:01Z</t>
+          <t>2026-10-22T12:51:05Z</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>morning-epi-overlap-backfill</t>
+          <t>evening-r4-figure-extract</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>include_core_overlap_backfill</t>
+          <t>apply_evening_r4e_uspto_figures</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>EPI-INCREMENTAL-SPRINT-morning-2026-10-22-frozen.json; EVIDENCE-MORNING-DIFF-2026-10-22 PASS_INCREMENTAL</t>
+          <t>US12770834B2+US12768074B2 drawing sheets; pubs=2; actually_read/research_through/team_read untouched by design</t>
         </is>
       </c>
     </row>
@@ -26238,7 +26234,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-US12768074B2</t>
+          <t>2026-10-US12770834B2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -26270,27 +26266,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-US12765027B2</t>
+          <t>2026-10-US12770834B2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-22T12:51:05Z</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-r4-figure-extract</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_uspto_drawing_sheet_figures</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Track A evening R4: 8 real USPTO drawing-sheet PNGs; team_read lock unchanged</t>
         </is>
       </c>
     </row>
@@ -26302,27 +26298,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-US20260313994A1</t>
+          <t>2026-10-US12768074B2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-22T01:54:01Z</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-epi-overlap-backfill</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_overlap_backfill</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>EPI-INCREMENTAL-SPRINT-morning-2026-10-22-frozen.json; EVIDENCE-MORNING-DIFF-2026-10-22 PASS_INCREMENTAL</t>
         </is>
       </c>
     </row>
@@ -26334,27 +26330,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-US12757647B2</t>
+          <t>2026-10-US12768074B2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-22T12:51:05Z</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-r4-figure-extract</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_uspto_drawing_sheet_figures</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Track A evening R4: 13 real USPTO drawing-sheet PNGs; team_read lock unchanged</t>
         </is>
       </c>
     </row>
@@ -26366,27 +26362,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-US12757648B2</t>
+          <t>2026-10-US12765027B2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-20T10:37:42Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>sprint-gap-a</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>content_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26398,27 +26394,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-US12757648B2</t>
+          <t>2026-10-US20260313994A1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26430,27 +26426,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-US12757665B2</t>
+          <t>2026-10-US12757647B2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>include_core_preclean_family</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -26462,27 +26458,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-US12757665B2</t>
+          <t>2026-10-US12757648B2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T10:37:42Z</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>sprint-gap-a</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>content_add</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Gate③ backfill 6 figures</t>
+          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
         </is>
       </c>
     </row>
@@ -26494,27 +26490,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-US20260304810A1</t>
+          <t>2026-10-US12757648B2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -26526,27 +26522,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-US12727402B2</t>
+          <t>2026-10-US12757665B2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_preclean_family</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -26558,27 +26554,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-US20260275525A1</t>
+          <t>2026-10-US12757665B2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 6 figures</t>
         </is>
       </c>
     </row>
@@ -26590,7 +26586,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-US20260282506A1</t>
+          <t>2026-10-US20260304810A1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -26622,7 +26618,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-US20260282794A1</t>
+          <t>2026-09-US12727402B2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -26654,7 +26650,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-US12745604B2</t>
+          <t>2026-09-US20260275525A1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -26686,7 +26682,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-US20260293620A1</t>
+          <t>2026-09-US20260282506A1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -26718,7 +26714,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-TWI939895B</t>
+          <t>2026-09-US20260282794A1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -26750,7 +26746,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-US12740346B2</t>
+          <t>2026-09-US12745604B2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -26782,7 +26778,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-US12698570B2</t>
+          <t>2026-09-US20260293620A1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -26814,7 +26810,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-US12701762B2</t>
+          <t>2026-09-TWI939895B</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -26846,7 +26842,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-US12707938B2</t>
+          <t>2026-09-US12740346B2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -26878,7 +26874,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-US20260250878A1</t>
+          <t>2026-08-US12698570B2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -26910,7 +26906,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-US12701931B2</t>
+          <t>2026-08-US12701762B2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -26942,7 +26938,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-US20260206272A1</t>
+          <t>2026-08-US12707938B2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -26974,7 +26970,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-US12692621B2</t>
+          <t>2026-08-US20260250878A1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -27006,7 +27002,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-US12696707B2</t>
+          <t>2026-08-US12701931B2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -27038,7 +27034,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-US12680191B2</t>
+          <t>2026-07-US20260206272A1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -27070,27 +27066,27 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-TW202628839A</t>
+          <t>2026-07-US12692621B2</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27102,27 +27098,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-TW202628839A</t>
+          <t>2026-07-US12696707B2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-20T10:50:56Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>preclean-figure-backfill</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27134,7 +27130,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-06-JP7882130B2</t>
+          <t>2026-07-US12680191B2</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -27166,27 +27162,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-06-US12672330B2</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27198,27 +27194,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-06-CN122294515A</t>
+          <t>2026-07-TW202628839A</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>preclean-figure-backfill</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
         </is>
       </c>
     </row>
@@ -27230,27 +27226,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-06-CN122294515A</t>
+          <t>2026-06-JP7882130B2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-20T13:05:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>preclean-cn-figure-stamp</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>attach_depats_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27262,7 +27258,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-06-US12655537B2</t>
+          <t>2026-06-US12672330B2</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -27294,27 +27290,27 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-06-US12660266B2</t>
+          <t>2026-06-CN122294515A</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27326,27 +27322,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-06-US12660522B2</t>
+          <t>2026-06-CN122294515A</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T13:05:00Z</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>preclean-cn-figure-stamp</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>attach_depats_figures</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
         </is>
       </c>
     </row>
@@ -27358,27 +27354,27 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-06-US12660522B2</t>
+          <t>2026-06-US12655537B2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27390,27 +27386,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-06-US12660544B2</t>
+          <t>2026-06-US12660266B2</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>include_core_preclean_family</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27422,27 +27418,27 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-06-US12660544B2</t>
+          <t>2026-06-US12660522B2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Gate③ backfill 6 figures</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27454,27 +27450,27 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-06-US20260164725A1</t>
+          <t>2026-06-US12660522B2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -27486,27 +27482,27 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-06-US12652840B2</t>
+          <t>2026-06-US12660544B2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_preclean_family</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -27518,27 +27514,27 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-06-US20260152871A1</t>
+          <t>2026-06-US12660544B2</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 6 figures</t>
         </is>
       </c>
     </row>
@@ -27550,7 +27546,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-05-US12628600B2</t>
+          <t>2026-06-US20260164725A1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -27582,7 +27578,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-06-US12652840B2</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -27614,27 +27610,27 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-05-US20260136521A1</t>
+          <t>2026-06-US20260152871A1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27646,7 +27642,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-05-US20260143977A1</t>
+          <t>2026-05-US12628600B2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -27678,7 +27674,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-05-WO2026101868A1</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -27710,27 +27706,27 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-05-US20260150594A1</t>
+          <t>2026-05-US20260136521A1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索对照命中。保留 reference_report 基线标记，不升级为独立新纳入。</t>
         </is>
       </c>
     </row>
@@ -27742,27 +27738,27 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-05-CN122069948A</t>
+          <t>2026-05-US20260143977A1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27774,27 +27770,27 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-05-CN122069948A</t>
+          <t>2026-05-WO2026101868A1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-20T13:05:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>preclean-cn-figure-stamp</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>attach_depats_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27806,27 +27802,27 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-05-WO2026096517A1</t>
+          <t>2026-05-US20260150594A1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -27838,27 +27834,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-05-WO2026096517A1</t>
+          <t>2026-05-CN122069948A</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-20T10:50:56Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>preclean-figure-backfill</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27870,27 +27866,27 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-04-US20260092399A1</t>
+          <t>2026-05-CN122069948A</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:05:00Z</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>preclean-cn-figure-stamp</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_depats_figures</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ Preclean CN DEPATISnet 附图 1–3（spotcheck PASS）</t>
         </is>
       </c>
     </row>
@@ -27902,27 +27898,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-04-JP2026512448A</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -27934,27 +27930,27 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-04-KR102954223B1</t>
+          <t>2026-05-WO2026096517A1</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T10:50:56Z</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>preclean-figure-backfill</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Applied 3 figures from PRECLEAN-REPORT-FIGURES-BACKFILL-2026-10-20.json</t>
         </is>
       </c>
     </row>
@@ -27966,7 +27962,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-04-WO2026079031A1</t>
+          <t>2026-04-US20260092399A1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -27998,7 +27994,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-04-WO2026084898A1</t>
+          <t>2026-04-JP2026512448A</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -28030,7 +28026,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-04-US20260123349A1</t>
+          <t>2026-04-KR102954223B1</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -28062,7 +28058,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-04-US12595587B2</t>
+          <t>2026-04-WO2026079031A1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -28094,7 +28090,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-03-JP2026510085A</t>
+          <t>2026-04-WO2026084898A1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -28126,7 +28122,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-03-US20260090293A1</t>
+          <t>2026-04-US20260123349A1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -28158,27 +28154,27 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-03-US20260090293A1</t>
+          <t>2026-04-US12595587B2</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>label_baseline_preclean_tag</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>US20260090293A1 已 live baseline；补 Preclean 技术标签（claim12），不计晚间新发现。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28190,7 +28186,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-03-KR20260039926A</t>
+          <t>2026-03-JP2026510085A</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -28222,27 +28218,27 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-03-CN121693111A</t>
+          <t>2026-03-US20260090293A1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28254,27 +28250,27 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-03-CN121693111A</t>
+          <t>2026-03-US20260090293A1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-20T12:50:00Z</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>epi-gate3-cn-figure-backfill</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>attach_fig1_depats</t>
+          <t>label_baseline_preclean_tag</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Official drawing page 1/3 → assets/figures/CN121693111A_fig1.png (08612a81…).</t>
+          <t>US20260090293A1 已 live baseline；补 Preclean 技术标签（claim12），不计晚间新发现。</t>
         </is>
       </c>
     </row>
@@ -28286,7 +28282,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-03-US20260076125A1</t>
+          <t>2026-03-KR20260039926A</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -28318,27 +28314,27 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-03-WO2026055216A1</t>
+          <t>2026-03-CN121693111A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -28350,27 +28346,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-03-US20260071979A1</t>
+          <t>2026-03-CN121693111A</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T12:50:00Z</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>epi-gate3-cn-figure-backfill</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>attach_fig1_depats</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Official drawing page 1/3 → assets/figures/CN121693111A_fig1.png (08612a81…).</t>
         </is>
       </c>
     </row>
@@ -28382,27 +28378,27 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-03-US20260071979A1</t>
+          <t>2026-03-US20260076125A1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28414,7 +28410,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-03-US20260068564A1</t>
+          <t>2026-03-WO2026055216A1</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -28446,27 +28442,27 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-03-US20260066234A1</t>
+          <t>2026-03-US20260071979A1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>read-ruling-r2</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>promote_core_team_read</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -28478,7 +28474,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-03-US20260066234A1</t>
+          <t>2026-03-US20260071979A1</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -28510,27 +28506,27 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-03-US20260062803A1</t>
+          <t>2026-03-US20260068564A1</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>include_core_epi</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>EPI-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28542,27 +28538,27 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-03-US20260062803A1</t>
+          <t>2026-03-US20260066234A1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T12:00:00Z</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>read-ruling-r2</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>promote_core_team_read</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Gate③ backfill 2 figures</t>
+          <t>由 pending 升格 core 月卡；不计为 Gate③ 独立新发现。</t>
         </is>
       </c>
     </row>
@@ -28574,27 +28570,27 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-02-US12540400B2</t>
+          <t>2026-03-US20260066234A1</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -28606,27 +28602,27 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-02-US20260043170A1</t>
+          <t>2026-03-US20260062803A1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_epi</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>EPI-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -28638,27 +28634,27 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-02-US20260047358A1</t>
+          <t>2026-03-US20260062803A1</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 2 figures</t>
         </is>
       </c>
     </row>
@@ -28670,7 +28666,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-02-WO2026035639A1</t>
+          <t>2026-02-US12540400B2</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -28702,7 +28698,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-02-CN121519154A</t>
+          <t>2026-02-US20260043170A1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -28734,7 +28730,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-02-US12557185B2</t>
+          <t>2026-02-US20260047358A1</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -28766,7 +28762,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-02-US20260049767A1</t>
+          <t>2026-02-WO2026035639A1</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -28798,7 +28794,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-02-US12564001B2</t>
+          <t>2026-02-CN121519154A</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -28830,7 +28826,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-US12557185B2</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -28862,27 +28858,27 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-02-US12543516B2</t>
+          <t>2026-02-US20260049767A1</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28894,7 +28890,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-02-US20260035835A1</t>
+          <t>2026-02-US12564001B2</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -28926,27 +28922,27 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-02-US20260055532A1</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -28958,27 +28954,27 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-02-US20260055532A1</t>
+          <t>2026-02-US12543516B2</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>独立检索对照命中。保留基线导入属性，仅记录对照复核。</t>
         </is>
       </c>
     </row>
@@ -28990,7 +28986,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-01-WO2026024419A1</t>
+          <t>2026-02-US20260035835A1</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -29022,27 +29018,27 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-01-KR102918757B1</t>
+          <t>2026-02-US20260055532A1</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -29054,27 +29050,27 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-01-WO2026016396A1</t>
+          <t>2026-02-US20260055532A1</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -29086,7 +29082,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-01-US20260026275A1</t>
+          <t>2026-01-WO2026024419A1</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -29118,7 +29114,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-01-KR102915695B1</t>
+          <t>2026-01-KR102918757B1</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -29150,27 +29146,27 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-01-KR102916044B1</t>
+          <t>2026-01-WO2026016396A1</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-20T13:00:00Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>evening-incremental-sprint</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>include_core_preclean_family</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -29182,27 +29178,27 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-01-KR102916044B1</t>
+          <t>2026-01-US20260026275A1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Gate③ backfill 6 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -29214,7 +29210,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-01-US20260015766A1</t>
+          <t>2026-01-KR102915695B1</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -29246,27 +29242,27 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-01-KR102916044B1</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T13:00:00Z</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evening-incremental-sprint</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>include_core_preclean_family</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>PRECLEAN-INCREMENTAL-SPRINT-evening-2026-10-20-frozen.json</t>
         </is>
       </c>
     </row>
@@ -29278,27 +29274,27 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-01-US12526971B2</t>
+          <t>2026-01-KR102916044B1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>independent_search_confirm</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
+          <t>Gate③ backfill 6 figures</t>
         </is>
       </c>
     </row>
@@ -29310,7 +29306,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-01-US20260009155A1</t>
+          <t>2026-01-US20260015766A1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -29342,7 +29338,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-01-WO2026005974A1</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -29374,27 +29370,27 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2025-12-KR20250168533A</t>
+          <t>2026-01-US12526971B2</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_search_confirm</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立 EPI 检索再次命中本条（2026-01 授权）。仅作对照确认，仍计为基线导入（imported baseline），不记为本团队新发现。</t>
         </is>
       </c>
     </row>
@@ -29406,7 +29402,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2025-12-US20250379096A1</t>
+          <t>2026-01-US20260009155A1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -29438,7 +29434,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2025-12-US20250385089A1</t>
+          <t>2026-01-WO2026005974A1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -29470,7 +29466,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2025-12-US20250385122A1</t>
+          <t>2025-12-KR20250168533A</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -29502,7 +29498,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2025-12-US12503791B2</t>
+          <t>2025-12-US20250379096A1</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -29534,7 +29530,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2025-12-KR102904356B1</t>
+          <t>2025-12-US20250385089A1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -29566,7 +29562,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2025-12-WO2025260942A1</t>
+          <t>2025-12-US20250385122A1</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -29598,7 +29594,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2025-12-US12512362B2</t>
+          <t>2025-12-US12503791B2</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -29630,7 +29626,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2025-12-US20250369154A1</t>
+          <t>2025-12-KR102904356B1</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -29662,7 +29658,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2025-11-KR102886069B1</t>
+          <t>2025-12-WO2025260942A1</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -29694,7 +29690,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2025-11-US20250351329A1</t>
+          <t>2025-12-US12512362B2</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -29726,7 +29722,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2025-11-WO2025232199A1</t>
+          <t>2025-12-US20250369154A1</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -29758,7 +29754,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2025-11-TW202544883A</t>
+          <t>2025-11-KR102886069B1</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -29790,7 +29786,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2025-11-KR102888301B1</t>
+          <t>2025-11-US20250351329A1</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -29822,7 +29818,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2025-11-US20250358906A1</t>
+          <t>2025-11-WO2025232199A1</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -29854,7 +29850,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2025-11-CN120989593A</t>
+          <t>2025-11-TW202544883A</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -29886,7 +29882,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2025-11-CN121002222A</t>
+          <t>2025-11-KR102888301B1</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -29918,7 +29914,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2025-11-CN121002231A</t>
+          <t>2025-11-US20250358906A1</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -29950,7 +29946,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2025-11-CN121002616A</t>
+          <t>2025-11-CN120989593A</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -29982,7 +29978,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2025-11-CN121002621A</t>
+          <t>2025-11-CN121002222A</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -30014,7 +30010,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2025-11-KR102889785B1</t>
+          <t>2025-11-CN121002231A</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -30046,7 +30042,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2025-11-TWI905596B</t>
+          <t>2025-11-CN121002616A</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -30078,7 +30074,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2025-11-CN223598701U</t>
+          <t>2025-11-CN121002621A</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -30110,7 +30106,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2025-11-US12480223B2</t>
+          <t>2025-11-KR102889785B1</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -30142,7 +30138,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2025-11-US12482662B2</t>
+          <t>2025-11-TWI905596B</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -30174,7 +30170,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2025-11-US12484327B2</t>
+          <t>2025-11-CN223598701U</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -30206,7 +30202,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2025-11-JP7776424B2</t>
+          <t>2025-11-US12480223B2</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -30238,7 +30234,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2025-11-DE112021001213B4</t>
+          <t>2025-11-US12482662B2</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -30270,7 +30266,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2025-11-WO2025244833A1</t>
+          <t>2025-11-US12484327B2</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -30302,7 +30298,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2025-10-WO2025225316A1</t>
+          <t>2025-11-JP7776424B2</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -30334,7 +30330,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2025-10-WO2025222891A1</t>
+          <t>2025-11-DE112021001213B4</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -30366,7 +30362,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2025-10-US12454769B2</t>
+          <t>2025-11-WO2025244833A1</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -30398,7 +30394,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2025-10-US20250327211A1</t>
+          <t>2025-10-WO2025225316A1</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -30430,7 +30426,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2025-10-WO2025220436A1</t>
+          <t>2025-10-WO2025222891A1</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -30462,7 +30458,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2025-10-WO2025221932A1</t>
+          <t>2025-10-US12454769B2</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -30494,7 +30490,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2025-10-US20250331222A1</t>
+          <t>2025-10-US20250327211A1</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -30526,27 +30522,27 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2025-10-US20250327209A1</t>
+          <t>2025-10-WO2025220436A1</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-20T09:31:48Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>evidence-review-r2</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>independent_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>独立检索新纳入（非基线导入）。</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -30558,27 +30554,27 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2025-10-US20250327209A1</t>
+          <t>2025-10-WO2025221932A1</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-21T02:07:37Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>morning-gate3-figures</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>attach_gate3_family_figures</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Gate③ backfill 1 figures</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -30590,7 +30586,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2025-10-JP7757917B2</t>
+          <t>2025-10-US20250331222A1</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -30622,27 +30618,27 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2025-10-KR20250150601A</t>
+          <t>2025-10-US20250327209A1</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-20T09:31:48Z</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>evidence-review-r2</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>independent_add</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>独立检索新纳入（非基线导入）。</t>
         </is>
       </c>
     </row>
@@ -30654,27 +30650,27 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2025-10-CN120797198A</t>
+          <t>2025-10-US20250327209A1</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-20T17:30:00+08:00</t>
+          <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>baseline-import</t>
+          <t>morning-gate3-figures</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>attach_gate3_family_figures</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+          <t>Gate③ backfill 1 figures</t>
         </is>
       </c>
     </row>
@@ -30686,7 +30682,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2025-10-US20250324699A1</t>
+          <t>2025-10-JP7757917B2</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -30718,7 +30714,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2025-10-US12444605B2</t>
+          <t>2025-10-KR20250150601A</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -30750,7 +30746,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2025-10-KR102870814B1</t>
+          <t>2025-10-CN120797198A</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -30782,7 +30778,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2025-10-WO2025211045A1</t>
+          <t>2025-10-US20250324699A1</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -30814,7 +30810,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2025-10-JP2025533523A</t>
+          <t>2025-10-US12444605B2</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -30846,7 +30842,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2025-10-WO2025204274A1</t>
+          <t>2025-10-KR102870814B1</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -30878,27 +30874,27 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2025-10-US20250311241A1</t>
+          <t>2025-10-WO2025211045A1</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-20T10:37:42Z</t>
+          <t>2026-10-20T17:30:00+08:00</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>sprint-gap-a</t>
+          <t>baseline-import</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>content_add</t>
+          <t>import</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
         </is>
       </c>
     </row>
@@ -30910,25 +30906,121 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
+          <t>2025-10-JP2025533523A</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2025-10-WO2025204274A1</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:30:00+08:00</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>baseline-import</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Imported from Dot reference report; not this team's independent discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
           <t>2025-10-US20250311241A1</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>2026-10-20T10:37:42Z</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>sprint-gap-a</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>content_add</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>EVIDENCE-SPRINT-A / EPI-INCREMENTAL-SPRINT-gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2025-10-US20250311241A1</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
         <is>
           <t>2026-10-21T02:07:37Z</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr">
+      <c r="D170" t="inlineStr">
         <is>
           <t>morning-gate3-figures</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr">
+      <c r="E170" t="inlineStr">
         <is>
           <t>attach_gate3_family_figures</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
+      <c r="F170" t="inlineStr">
         <is>
           <t>Gate③ backfill 1 figures</t>
         </is>

</xml_diff>